<commit_message>
Rates update 2026-10-20 23:33 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Daily Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="History" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="History" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -582,11 +582,11 @@
         <v>11085</v>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-20 22:41:20</t>
+          <t>2026-10-20 23:33:51</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2108,6 +2108,150 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-10-20 23:33:51</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>14717</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>-87</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-10-20 23:33:51</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>13490</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>-80</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-10-20 23:33:51</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>11085</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>-70</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-20 23:40 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -582,11 +582,11 @@
         <v>11085</v>
       </c>
       <c r="O2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-20 23:33:51</t>
+          <t>2026-10-20 23:40:06</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2252,6 +2252,150 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-10-20 23:40:06</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>14717</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>-87</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-10-20 23:40:06</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>13490</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>-80</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-10-20 23:40:06</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>11085</v>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>-70</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-21 16:49 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -546,54 +546,54 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-87</v>
+        <v>-109</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-80</v>
+        <v>-100</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>-70</v>
+        <v>-115</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="O2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-20 23:40:06</t>
+          <t>2026-10-21 16:49:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -602,46 +602,54 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="E3" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="F3" s="3" t="n">
-        <v>38</v>
+        <v>-87</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="H3" s="3" t="n"/>
+        <v>-80</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>-70</v>
+      </c>
       <c r="I3" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="K3" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="L3" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="N3" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="O3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-10-19 00:00:00</t>
+          <t>2026-10-20 23:40:06</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -650,31 +658,31 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="E4" s="2" t="n"/>
       <c r="F4" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H4" s="3" t="n"/>
       <c r="I4" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="K4" s="2" t="n"/>
       <c r="L4" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="N4" s="2" t="n"/>
       <c r="O4" t="n">
@@ -682,14 +690,14 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-10-18 00:00:00</t>
+          <t>2026-10-19 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -705,10 +713,10 @@
       </c>
       <c r="E5" s="2" t="n"/>
       <c r="F5" s="3" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="2" t="n">
@@ -730,14 +738,14 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-10-17 00:00:00</t>
+          <t>2026-10-18 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -746,31 +754,31 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="E6" s="2" t="n"/>
       <c r="F6" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H6" s="3" t="n"/>
       <c r="I6" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="N6" s="2" t="n"/>
       <c r="O6" t="n">
@@ -778,14 +786,14 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-10-16 00:00:00</t>
+          <t>2026-10-17 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -801,10 +809,10 @@
       </c>
       <c r="E7" s="2" t="n"/>
       <c r="F7" s="3" t="n">
-        <v>-82</v>
+        <v>0</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-75</v>
+        <v>0</v>
       </c>
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="2" t="n">
@@ -826,14 +834,14 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-16 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -842,31 +850,31 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="3" t="n">
-        <v>-103</v>
+        <v>-82</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-95</v>
+        <v>-75</v>
       </c>
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="K8" s="2" t="n"/>
       <c r="L8" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="N8" s="2" t="n"/>
       <c r="O8" t="n">
@@ -874,14 +882,14 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -890,31 +898,31 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="3" t="n">
-        <v>-39</v>
+        <v>-103</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>-35</v>
+        <v>-95</v>
       </c>
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="K9" s="2" t="n"/>
       <c r="L9" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="N9" s="2" t="n"/>
       <c r="O9" t="n">
@@ -922,14 +930,14 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -938,31 +946,31 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="3" t="n">
-        <v>-174</v>
+        <v>-39</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-160</v>
+        <v>-35</v>
       </c>
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="K10" s="2" t="n"/>
       <c r="L10" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="N10" s="2" t="n"/>
       <c r="O10" t="n">
@@ -970,14 +978,14 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-10-12 00:00:00</t>
+          <t>2026-10-13 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -986,37 +994,85 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="3" t="n">
-        <v>0</v>
+        <v>-174</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0</v>
+        <v>-160</v>
       </c>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="N11" s="2" t="n"/>
       <c r="O11" t="n">
         <v>1</v>
       </c>
       <c r="P11" t="inlineStr">
+        <is>
+          <t>2026-10-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="K12" s="2" t="n"/>
+      <c r="L12" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="N12" s="2" t="n"/>
+      <c r="O12" t="n">
+        <v>1</v>
+      </c>
+      <c r="P12" t="inlineStr">
         <is>
           <t>2026-10-11 00:00:00</t>
         </is>
@@ -1033,7 +1089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2396,6 +2452,150 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-10-21 16:49:07</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>14608</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>-109</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-10-21 16:49:07</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>13390</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>-100</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-10-21 16:49:07</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>10970</v>
+      </c>
+      <c r="H31" s="3" t="n">
+        <v>-115</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-21 20:04 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -582,11 +582,11 @@
         <v>10970</v>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-21 16:49:07</t>
+          <t>2026-10-21 20:04:26</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2596,6 +2596,150 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-10-21 20:04:26</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>14608</v>
+      </c>
+      <c r="H32" s="3" t="n">
+        <v>-109</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-10-21 20:04:26</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>13390</v>
+      </c>
+      <c r="H33" s="3" t="n">
+        <v>-100</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-10-21 20:04:26</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>10970</v>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>-115</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-22 16:48 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -546,54 +546,54 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-109</v>
+        <v>-170</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-100</v>
+        <v>-155</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>-115</v>
+        <v>-135</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="O2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-21 20:04:26</t>
+          <t>2026-10-22 16:48:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -602,54 +602,54 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>-87</v>
+        <v>-109</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>-80</v>
+        <v>-100</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>-70</v>
+        <v>-115</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="O3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-10-20 23:40:06</t>
+          <t>2026-10-21 20:04:26</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -658,46 +658,54 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="E4" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="F4" s="3" t="n">
-        <v>38</v>
+        <v>-87</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="H4" s="3" t="n"/>
+        <v>-80</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>-70</v>
+      </c>
       <c r="I4" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="K4" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="L4" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="N4" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="O4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-10-19 00:00:00</t>
+          <t>2026-10-20 23:40:06</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -706,31 +714,31 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="E5" s="2" t="n"/>
       <c r="F5" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="N5" s="2" t="n"/>
       <c r="O5" t="n">
@@ -738,14 +746,14 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-10-18 00:00:00</t>
+          <t>2026-10-19 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -761,10 +769,10 @@
       </c>
       <c r="E6" s="2" t="n"/>
       <c r="F6" s="3" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H6" s="3" t="n"/>
       <c r="I6" s="2" t="n">
@@ -786,14 +794,14 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-10-17 00:00:00</t>
+          <t>2026-10-18 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -802,31 +810,31 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="E7" s="2" t="n"/>
       <c r="F7" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="K7" s="2" t="n"/>
       <c r="L7" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="N7" s="2" t="n"/>
       <c r="O7" t="n">
@@ -834,14 +842,14 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-10-16 00:00:00</t>
+          <t>2026-10-17 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -857,10 +865,10 @@
       </c>
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="3" t="n">
-        <v>-82</v>
+        <v>0</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-75</v>
+        <v>0</v>
       </c>
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="2" t="n">
@@ -882,14 +890,14 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-16 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -898,31 +906,31 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="3" t="n">
-        <v>-103</v>
+        <v>-82</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>-95</v>
+        <v>-75</v>
       </c>
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="K9" s="2" t="n"/>
       <c r="L9" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="N9" s="2" t="n"/>
       <c r="O9" t="n">
@@ -930,14 +938,14 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -946,31 +954,31 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="3" t="n">
-        <v>-39</v>
+        <v>-103</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-35</v>
+        <v>-95</v>
       </c>
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="K10" s="2" t="n"/>
       <c r="L10" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="N10" s="2" t="n"/>
       <c r="O10" t="n">
@@ -978,14 +986,14 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -994,31 +1002,31 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="3" t="n">
-        <v>-174</v>
+        <v>-39</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>-160</v>
+        <v>-35</v>
       </c>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="N11" s="2" t="n"/>
       <c r="O11" t="n">
@@ -1026,14 +1034,14 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-10-12 00:00:00</t>
+          <t>2026-10-13 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1042,37 +1050,85 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="3" t="n">
-        <v>0</v>
+        <v>-174</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0</v>
+        <v>-160</v>
       </c>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="N12" s="2" t="n"/>
       <c r="O12" t="n">
         <v>1</v>
       </c>
       <c r="P12" t="inlineStr">
+        <is>
+          <t>2026-10-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="N13" s="2" t="n"/>
+      <c r="O13" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" t="inlineStr">
         <is>
           <t>2026-10-11 00:00:00</t>
         </is>
@@ -1089,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2740,6 +2796,150 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-10-22 16:48:19</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>14438</v>
+      </c>
+      <c r="H35" s="3" t="n">
+        <v>-170</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-10-22 16:48:19</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>13235</v>
+      </c>
+      <c r="H36" s="3" t="n">
+        <v>-155</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-10-22 16:48:19</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>10835</v>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>-135</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-22 20:06 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -582,11 +582,11 @@
         <v>10835</v>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-22 16:48:19</t>
+          <t>2026-10-22 20:06:02</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2940,6 +2940,150 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-10-22 20:06:02</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>14438</v>
+      </c>
+      <c r="H38" s="3" t="n">
+        <v>-170</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-10-22 20:06:02</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>13235</v>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>-155</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-10-22 20:06:02</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>10835</v>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>-135</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-23 16:39 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -546,54 +546,54 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-170</v>
+        <v>-190</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-155</v>
+        <v>-175</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>-135</v>
+        <v>-145</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="O2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-22 20:06:02</t>
+          <t>2026-10-23 16:39:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -602,54 +602,54 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>-109</v>
+        <v>-170</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>-100</v>
+        <v>-155</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>-115</v>
+        <v>-135</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="O3" t="n">
         <v>2</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-10-21 20:04:26</t>
+          <t>2026-10-22 20:06:02</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -658,54 +658,54 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>-87</v>
+        <v>-109</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>-80</v>
+        <v>-100</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>-70</v>
+        <v>-115</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="O4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-10-20 23:40:06</t>
+          <t>2026-10-21 20:04:26</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -714,46 +714,54 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="E5" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="F5" s="3" t="n">
-        <v>38</v>
+        <v>-87</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="H5" s="3" t="n"/>
+        <v>-80</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>-70</v>
+      </c>
       <c r="I5" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="K5" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="L5" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="N5" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="O5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-10-19 00:00:00</t>
+          <t>2026-10-20 23:40:06</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -762,31 +770,31 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="E6" s="2" t="n"/>
       <c r="F6" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H6" s="3" t="n"/>
       <c r="I6" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="N6" s="2" t="n"/>
       <c r="O6" t="n">
@@ -794,14 +802,14 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-10-18 00:00:00</t>
+          <t>2026-10-19 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -817,10 +825,10 @@
       </c>
       <c r="E7" s="2" t="n"/>
       <c r="F7" s="3" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="2" t="n">
@@ -842,14 +850,14 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-10-17 00:00:00</t>
+          <t>2026-10-18 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -858,31 +866,31 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="K8" s="2" t="n"/>
       <c r="L8" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="N8" s="2" t="n"/>
       <c r="O8" t="n">
@@ -890,14 +898,14 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-10-16 00:00:00</t>
+          <t>2026-10-17 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -913,10 +921,10 @@
       </c>
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="3" t="n">
-        <v>-82</v>
+        <v>0</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>-75</v>
+        <v>0</v>
       </c>
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="2" t="n">
@@ -938,14 +946,14 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-16 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -954,31 +962,31 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="3" t="n">
-        <v>-103</v>
+        <v>-82</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-95</v>
+        <v>-75</v>
       </c>
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="K10" s="2" t="n"/>
       <c r="L10" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="N10" s="2" t="n"/>
       <c r="O10" t="n">
@@ -986,14 +994,14 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1002,31 +1010,31 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="3" t="n">
-        <v>-39</v>
+        <v>-103</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>-35</v>
+        <v>-95</v>
       </c>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="N11" s="2" t="n"/>
       <c r="O11" t="n">
@@ -1034,14 +1042,14 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1050,31 +1058,31 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="3" t="n">
-        <v>-174</v>
+        <v>-39</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-160</v>
+        <v>-35</v>
       </c>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="N12" s="2" t="n"/>
       <c r="O12" t="n">
@@ -1082,14 +1090,14 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2026-10-12 00:00:00</t>
+          <t>2026-10-13 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1098,37 +1106,85 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="E13" s="2" t="n"/>
       <c r="F13" s="3" t="n">
-        <v>0</v>
+        <v>-174</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>0</v>
+        <v>-160</v>
       </c>
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="N13" s="2" t="n"/>
       <c r="O13" t="n">
         <v>1</v>
       </c>
       <c r="P13" t="inlineStr">
+        <is>
+          <t>2026-10-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="3" t="n"/>
+      <c r="I14" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="K14" s="2" t="n"/>
+      <c r="L14" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="N14" s="2" t="n"/>
+      <c r="O14" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" t="inlineStr">
         <is>
           <t>2026-10-11 00:00:00</t>
         </is>
@@ -1145,7 +1201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3084,6 +3140,150 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-10-23 16:39:12</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>14248</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>-190</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-10-23 16:39:12</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>13060</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>-175</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-10-23 16:39:12</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>10690</v>
+      </c>
+      <c r="H43" s="3" t="n">
+        <v>-145</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-23 19:50 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -582,11 +582,11 @@
         <v>10690</v>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-23 16:39:12</t>
+          <t>2026-10-23 19:50:04</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3284,6 +3284,150 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-10-23 19:50:04</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>14248</v>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>-190</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-10-23 19:50:04</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>13060</v>
+      </c>
+      <c r="H45" s="3" t="n">
+        <v>-175</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-10-23 19:50:04</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>10690</v>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>-145</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-24 15:56 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -546,54 +546,54 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-190</v>
+        <v>10</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-175</v>
+        <v>10</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>-145</v>
+        <v>5</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="O2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:04</t>
+          <t>2026-10-24 15:56:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -602,54 +602,54 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>-170</v>
+        <v>-190</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>-155</v>
+        <v>-175</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>-135</v>
+        <v>-145</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="O3" t="n">
         <v>2</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-10-22 20:06:02</t>
+          <t>2026-10-23 19:50:04</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -658,54 +658,54 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>-109</v>
+        <v>-170</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>-100</v>
+        <v>-155</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>-115</v>
+        <v>-135</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="O4" t="n">
         <v>2</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-10-21 20:04:26</t>
+          <t>2026-10-22 20:06:02</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -714,54 +714,54 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>-87</v>
+        <v>-109</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-80</v>
+        <v>-100</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>-70</v>
+        <v>-115</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="O5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-10-20 23:40:06</t>
+          <t>2026-10-21 20:04:26</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -770,46 +770,54 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="E6" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="F6" s="3" t="n">
-        <v>38</v>
+        <v>-87</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="H6" s="3" t="n"/>
+        <v>-80</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>-70</v>
+      </c>
       <c r="I6" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="K6" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="L6" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="N6" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="O6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-10-19 00:00:00</t>
+          <t>2026-10-20 23:40:06</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -818,31 +826,31 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="E7" s="2" t="n"/>
       <c r="F7" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="K7" s="2" t="n"/>
       <c r="L7" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="N7" s="2" t="n"/>
       <c r="O7" t="n">
@@ -850,14 +858,14 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-10-18 00:00:00</t>
+          <t>2026-10-19 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -873,10 +881,10 @@
       </c>
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="3" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="2" t="n">
@@ -898,14 +906,14 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-10-17 00:00:00</t>
+          <t>2026-10-18 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -914,31 +922,31 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="K9" s="2" t="n"/>
       <c r="L9" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="N9" s="2" t="n"/>
       <c r="O9" t="n">
@@ -946,14 +954,14 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-10-16 00:00:00</t>
+          <t>2026-10-17 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -969,10 +977,10 @@
       </c>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="3" t="n">
-        <v>-82</v>
+        <v>0</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-75</v>
+        <v>0</v>
       </c>
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="2" t="n">
@@ -994,14 +1002,14 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-16 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1010,31 +1018,31 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="3" t="n">
-        <v>-103</v>
+        <v>-82</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>-95</v>
+        <v>-75</v>
       </c>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="N11" s="2" t="n"/>
       <c r="O11" t="n">
@@ -1042,14 +1050,14 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1058,31 +1066,31 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="3" t="n">
-        <v>-39</v>
+        <v>-103</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-35</v>
+        <v>-95</v>
       </c>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="N12" s="2" t="n"/>
       <c r="O12" t="n">
@@ -1090,14 +1098,14 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1106,31 +1114,31 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="E13" s="2" t="n"/>
       <c r="F13" s="3" t="n">
-        <v>-174</v>
+        <v>-39</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-160</v>
+        <v>-35</v>
       </c>
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="N13" s="2" t="n"/>
       <c r="O13" t="n">
@@ -1138,14 +1146,14 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2026-10-12 00:00:00</t>
+          <t>2026-10-13 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1154,37 +1162,85 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="3" t="n">
-        <v>0</v>
+        <v>-174</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>0</v>
+        <v>-160</v>
       </c>
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="N14" s="2" t="n"/>
       <c r="O14" t="n">
         <v>1</v>
       </c>
       <c r="P14" t="inlineStr">
+        <is>
+          <t>2026-10-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="K15" s="2" t="n"/>
+      <c r="L15" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="N15" s="2" t="n"/>
+      <c r="O15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P15" t="inlineStr">
         <is>
           <t>2026-10-11 00:00:00</t>
         </is>
@@ -1201,7 +1257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3428,6 +3484,150 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-10-24 15:56:21</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>14258</v>
+      </c>
+      <c r="H47" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-10-24 15:56:21</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>13070</v>
+      </c>
+      <c r="H48" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-10-24 15:56:21</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>10695</v>
+      </c>
+      <c r="H49" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-24 18:57 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -582,11 +582,11 @@
         <v>10695</v>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-24 15:56:21</t>
+          <t>2026-10-24 18:56:58</t>
         </is>
       </c>
     </row>
@@ -1257,7 +1257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3628,6 +3628,150 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-10-24 18:56:58</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>14258</v>
+      </c>
+      <c r="H50" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-10-24 18:56:58</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>13070</v>
+      </c>
+      <c r="H51" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-10-24 18:56:58</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>10695</v>
+      </c>
+      <c r="H52" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-25 16:23 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -554,15 +554,9 @@
       <c r="E2" s="2" t="n">
         <v>10695</v>
       </c>
-      <c r="F2" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H2" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
       <c r="I2" s="2" t="n">
         <v>14258</v>
       </c>
@@ -582,18 +576,18 @@
         <v>10695</v>
       </c>
       <c r="O2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-24 18:56:58</t>
+          <t>2026-10-25 16:23:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -602,54 +596,54 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>-190</v>
+        <v>10</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>-175</v>
+        <v>10</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>-145</v>
+        <v>5</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="O3" t="n">
         <v>2</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:04</t>
+          <t>2026-10-24 18:56:58</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -658,54 +652,54 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>-170</v>
+        <v>-190</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>-155</v>
+        <v>-175</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>-135</v>
+        <v>-145</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="O4" t="n">
         <v>2</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-10-22 20:06:02</t>
+          <t>2026-10-23 19:50:04</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -714,54 +708,54 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>-109</v>
+        <v>-170</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-100</v>
+        <v>-155</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>-115</v>
+        <v>-135</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="O5" t="n">
         <v>2</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-10-21 20:04:26</t>
+          <t>2026-10-22 20:06:02</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -770,54 +764,54 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-87</v>
+        <v>-109</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-80</v>
+        <v>-100</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>-70</v>
+        <v>-115</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="O6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-10-20 23:40:06</t>
+          <t>2026-10-21 20:04:26</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -826,46 +820,54 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="E7" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="F7" s="3" t="n">
-        <v>38</v>
+        <v>-87</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="H7" s="3" t="n"/>
+        <v>-80</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>-70</v>
+      </c>
       <c r="I7" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="K7" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="L7" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="N7" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="O7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-10-19 00:00:00</t>
+          <t>2026-10-20 23:40:06</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -874,31 +876,31 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="K8" s="2" t="n"/>
       <c r="L8" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="N8" s="2" t="n"/>
       <c r="O8" t="n">
@@ -906,14 +908,14 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-10-18 00:00:00</t>
+          <t>2026-10-19 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -929,10 +931,10 @@
       </c>
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="3" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="2" t="n">
@@ -954,14 +956,14 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-10-17 00:00:00</t>
+          <t>2026-10-18 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -970,31 +972,31 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="K10" s="2" t="n"/>
       <c r="L10" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="N10" s="2" t="n"/>
       <c r="O10" t="n">
@@ -1002,14 +1004,14 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-10-16 00:00:00</t>
+          <t>2026-10-17 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1025,10 +1027,10 @@
       </c>
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="3" t="n">
-        <v>-82</v>
+        <v>0</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>-75</v>
+        <v>0</v>
       </c>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="2" t="n">
@@ -1050,14 +1052,14 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-16 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1066,31 +1068,31 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="3" t="n">
-        <v>-103</v>
+        <v>-82</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-95</v>
+        <v>-75</v>
       </c>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="N12" s="2" t="n"/>
       <c r="O12" t="n">
@@ -1098,14 +1100,14 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1114,31 +1116,31 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="E13" s="2" t="n"/>
       <c r="F13" s="3" t="n">
-        <v>-39</v>
+        <v>-103</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-35</v>
+        <v>-95</v>
       </c>
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="N13" s="2" t="n"/>
       <c r="O13" t="n">
@@ -1146,14 +1148,14 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1162,31 +1164,31 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="3" t="n">
-        <v>-174</v>
+        <v>-39</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>-160</v>
+        <v>-35</v>
       </c>
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="N14" s="2" t="n"/>
       <c r="O14" t="n">
@@ -1194,14 +1196,14 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2026-10-12 00:00:00</t>
+          <t>2026-10-13 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1210,37 +1212,85 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="3" t="n">
-        <v>0</v>
+        <v>-174</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>0</v>
+        <v>-160</v>
       </c>
       <c r="H15" s="3" t="n"/>
       <c r="I15" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="N15" s="2" t="n"/>
       <c r="O15" t="n">
         <v>1</v>
       </c>
       <c r="P15" t="inlineStr">
+        <is>
+          <t>2026-10-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="3" t="n"/>
+      <c r="I16" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="N16" s="2" t="n"/>
+      <c r="O16" t="n">
+        <v>1</v>
+      </c>
+      <c r="P16" t="inlineStr">
         <is>
           <t>2026-10-11 00:00:00</t>
         </is>
@@ -1257,7 +1307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3772,6 +3822,144 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-10-25 16:23:10</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>14258</v>
+      </c>
+      <c r="H53" s="3" t="n"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-10-25 16:23:10</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>13070</v>
+      </c>
+      <c r="H54" s="3" t="n"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-10-25 16:23:10</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>10695</v>
+      </c>
+      <c r="H55" s="3" t="n"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-25 19:18 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -576,11 +576,11 @@
         <v>10695</v>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-25 16:23:10</t>
+          <t>2026-10-25 19:18:46</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3960,6 +3960,144 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-10-25 19:18:46</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>14258</v>
+      </c>
+      <c r="H56" s="3" t="n"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-10-25 19:18:46</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>13070</v>
+      </c>
+      <c r="H57" s="3" t="n"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-10-25 19:18:46</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>10695</v>
+      </c>
+      <c r="H58" s="3" t="n"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-26 17:54 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -546,48 +546,54 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>10695</v>
-      </c>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
+        <v>10705</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="I2" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>10695</v>
+        <v>10705</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>10695</v>
+        <v>10705</v>
       </c>
       <c r="O2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-25 19:18:46</t>
+          <t>2026-10-26 17:54:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -604,15 +610,9 @@
       <c r="E3" s="2" t="n">
         <v>10695</v>
       </c>
-      <c r="F3" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
       <c r="I3" s="2" t="n">
         <v>14258</v>
       </c>
@@ -636,14 +636,14 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-10-24 18:56:58</t>
+          <t>2026-10-25 19:18:46</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -652,54 +652,54 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>-190</v>
+        <v>10</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>-175</v>
+        <v>10</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>-145</v>
+        <v>5</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="O4" t="n">
         <v>2</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:04</t>
+          <t>2026-10-24 18:56:58</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -708,54 +708,54 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>-170</v>
+        <v>-190</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-155</v>
+        <v>-175</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>-135</v>
+        <v>-145</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="O5" t="n">
         <v>2</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-10-22 20:06:02</t>
+          <t>2026-10-23 19:50:04</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -764,54 +764,54 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-109</v>
+        <v>-170</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-100</v>
+        <v>-155</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>-115</v>
+        <v>-135</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="O6" t="n">
         <v>2</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-10-21 20:04:26</t>
+          <t>2026-10-22 20:06:02</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -820,54 +820,54 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-87</v>
+        <v>-109</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-80</v>
+        <v>-100</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>-70</v>
+        <v>-115</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="O7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-10-20 23:40:06</t>
+          <t>2026-10-21 20:04:26</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -876,46 +876,54 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="E8" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="F8" s="3" t="n">
-        <v>38</v>
+        <v>-87</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="H8" s="3" t="n"/>
+        <v>-80</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>-70</v>
+      </c>
       <c r="I8" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="K8" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="L8" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="N8" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="O8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-10-19 00:00:00</t>
+          <t>2026-10-20 23:40:06</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -924,31 +932,31 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="K9" s="2" t="n"/>
       <c r="L9" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="N9" s="2" t="n"/>
       <c r="O9" t="n">
@@ -956,14 +964,14 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-10-18 00:00:00</t>
+          <t>2026-10-19 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -979,10 +987,10 @@
       </c>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="3" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="2" t="n">
@@ -1004,14 +1012,14 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-10-17 00:00:00</t>
+          <t>2026-10-18 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1020,31 +1028,31 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="N11" s="2" t="n"/>
       <c r="O11" t="n">
@@ -1052,14 +1060,14 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-10-16 00:00:00</t>
+          <t>2026-10-17 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1075,10 +1083,10 @@
       </c>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="3" t="n">
-        <v>-82</v>
+        <v>0</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-75</v>
+        <v>0</v>
       </c>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="2" t="n">
@@ -1100,14 +1108,14 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-16 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1116,31 +1124,31 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="E13" s="2" t="n"/>
       <c r="F13" s="3" t="n">
-        <v>-103</v>
+        <v>-82</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-95</v>
+        <v>-75</v>
       </c>
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="N13" s="2" t="n"/>
       <c r="O13" t="n">
@@ -1148,14 +1156,14 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1164,31 +1172,31 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="3" t="n">
-        <v>-39</v>
+        <v>-103</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>-35</v>
+        <v>-95</v>
       </c>
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="N14" s="2" t="n"/>
       <c r="O14" t="n">
@@ -1196,14 +1204,14 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1212,31 +1220,31 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="3" t="n">
-        <v>-174</v>
+        <v>-39</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-160</v>
+        <v>-35</v>
       </c>
       <c r="H15" s="3" t="n"/>
       <c r="I15" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="N15" s="2" t="n"/>
       <c r="O15" t="n">
@@ -1244,14 +1252,14 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2026-10-12 00:00:00</t>
+          <t>2026-10-13 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1260,37 +1268,85 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="3" t="n">
-        <v>0</v>
+        <v>-174</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>0</v>
+        <v>-160</v>
       </c>
       <c r="H16" s="3" t="n"/>
       <c r="I16" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="N16" s="2" t="n"/>
       <c r="O16" t="n">
         <v>1</v>
       </c>
       <c r="P16" t="inlineStr">
+        <is>
+          <t>2026-10-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="N17" s="2" t="n"/>
+      <c r="O17" t="n">
+        <v>1</v>
+      </c>
+      <c r="P17" t="inlineStr">
         <is>
           <t>2026-10-11 00:00:00</t>
         </is>
@@ -1307,7 +1363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4098,6 +4154,150 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-10-26 17:54:19</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>14275</v>
+      </c>
+      <c r="H59" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-10-26 17:54:19</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>13085</v>
+      </c>
+      <c r="H60" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-10-26 17:54:19</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>10705</v>
+      </c>
+      <c r="H61" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-26 21:44 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -582,11 +582,11 @@
         <v>10705</v>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-26 17:54:19</t>
+          <t>2026-10-26 21:44:41</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4298,6 +4298,150 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-10-26 21:44:41</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>14275</v>
+      </c>
+      <c r="H62" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-10-26 21:44:41</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>13085</v>
+      </c>
+      <c r="H63" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-10-26 21:44:41</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>10705</v>
+      </c>
+      <c r="H64" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-27 17:13 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -546,54 +546,54 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>14275</v>
+        <v>14329</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>13085</v>
+        <v>13135</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>10705</v>
+        <v>10750</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>14275</v>
+        <v>14329</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>13085</v>
+        <v>13135</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>10705</v>
+        <v>10750</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>14275</v>
+        <v>14329</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>13085</v>
+        <v>13135</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>10705</v>
+        <v>10750</v>
       </c>
       <c r="O2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-26 21:44:41</t>
+          <t>2026-10-27 17:13:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -602,48 +602,54 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>10695</v>
-      </c>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
+        <v>10705</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="I3" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>10695</v>
+        <v>10705</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>10695</v>
+        <v>10705</v>
       </c>
       <c r="O3" t="n">
         <v>2</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-10-25 19:18:46</t>
+          <t>2026-10-26 21:44:41</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -660,15 +666,9 @@
       <c r="E4" s="2" t="n">
         <v>10695</v>
       </c>
-      <c r="F4" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
       <c r="I4" s="2" t="n">
         <v>14258</v>
       </c>
@@ -692,14 +692,14 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-10-24 18:56:58</t>
+          <t>2026-10-25 19:18:46</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -708,54 +708,54 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>-190</v>
+        <v>10</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-175</v>
+        <v>10</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>-145</v>
+        <v>5</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="O5" t="n">
         <v>2</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:04</t>
+          <t>2026-10-24 18:56:58</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -764,54 +764,54 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-170</v>
+        <v>-190</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-155</v>
+        <v>-175</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>-135</v>
+        <v>-145</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="O6" t="n">
         <v>2</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-10-22 20:06:02</t>
+          <t>2026-10-23 19:50:04</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -820,54 +820,54 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-109</v>
+        <v>-170</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-100</v>
+        <v>-155</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>-115</v>
+        <v>-135</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="O7" t="n">
         <v>2</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-10-21 20:04:26</t>
+          <t>2026-10-22 20:06:02</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -876,54 +876,54 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-87</v>
+        <v>-109</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-80</v>
+        <v>-100</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>-70</v>
+        <v>-115</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="O8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-10-20 23:40:06</t>
+          <t>2026-10-21 20:04:26</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -932,46 +932,54 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="E9" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="F9" s="3" t="n">
-        <v>38</v>
+        <v>-87</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="H9" s="3" t="n"/>
+        <v>-80</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>-70</v>
+      </c>
       <c r="I9" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="K9" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="L9" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="N9" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="O9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-10-19 00:00:00</t>
+          <t>2026-10-20 23:40:06</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -980,31 +988,31 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="K10" s="2" t="n"/>
       <c r="L10" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="N10" s="2" t="n"/>
       <c r="O10" t="n">
@@ -1012,14 +1020,14 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-10-18 00:00:00</t>
+          <t>2026-10-19 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1035,10 +1043,10 @@
       </c>
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="3" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="2" t="n">
@@ -1060,14 +1068,14 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-10-17 00:00:00</t>
+          <t>2026-10-18 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1076,31 +1084,31 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="N12" s="2" t="n"/>
       <c r="O12" t="n">
@@ -1108,14 +1116,14 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2026-10-16 00:00:00</t>
+          <t>2026-10-17 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1131,10 +1139,10 @@
       </c>
       <c r="E13" s="2" t="n"/>
       <c r="F13" s="3" t="n">
-        <v>-82</v>
+        <v>0</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-75</v>
+        <v>0</v>
       </c>
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="2" t="n">
@@ -1156,14 +1164,14 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-16 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1172,31 +1180,31 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="3" t="n">
-        <v>-103</v>
+        <v>-82</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>-95</v>
+        <v>-75</v>
       </c>
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="N14" s="2" t="n"/>
       <c r="O14" t="n">
@@ -1204,14 +1212,14 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1220,31 +1228,31 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="3" t="n">
-        <v>-39</v>
+        <v>-103</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-35</v>
+        <v>-95</v>
       </c>
       <c r="H15" s="3" t="n"/>
       <c r="I15" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="N15" s="2" t="n"/>
       <c r="O15" t="n">
@@ -1252,14 +1260,14 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1268,31 +1276,31 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="3" t="n">
-        <v>-174</v>
+        <v>-39</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>-160</v>
+        <v>-35</v>
       </c>
       <c r="H16" s="3" t="n"/>
       <c r="I16" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="N16" s="2" t="n"/>
       <c r="O16" t="n">
@@ -1300,14 +1308,14 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>2026-10-12 00:00:00</t>
+          <t>2026-10-13 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1316,37 +1324,85 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="3" t="n">
-        <v>0</v>
+        <v>-174</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>0</v>
+        <v>-160</v>
       </c>
       <c r="H17" s="3" t="n"/>
       <c r="I17" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="N17" s="2" t="n"/>
       <c r="O17" t="n">
         <v>1</v>
       </c>
       <c r="P17" t="inlineStr">
+        <is>
+          <t>2026-10-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="N18" s="2" t="n"/>
+      <c r="O18" t="n">
+        <v>1</v>
+      </c>
+      <c r="P18" t="inlineStr">
         <is>
           <t>2026-10-11 00:00:00</t>
         </is>
@@ -1363,7 +1419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4442,6 +4498,150 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-10-27 17:13:22</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>14329</v>
+      </c>
+      <c r="H65" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-10-27 17:13:22</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>13135</v>
+      </c>
+      <c r="H66" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-10-27 17:13:22</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>10750</v>
+      </c>
+      <c r="H67" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-27 20:58 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -582,11 +582,11 @@
         <v>10750</v>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:13:22</t>
+          <t>2026-10-27 20:58:49</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J67"/>
+  <dimension ref="A1:J70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4642,6 +4642,150 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-10-27 20:58:49</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>14329</v>
+      </c>
+      <c r="H68" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-10-27 20:58:49</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>13135</v>
+      </c>
+      <c r="H69" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-10-27 20:58:49</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>10750</v>
+      </c>
+      <c r="H70" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-28 17:46 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -546,54 +546,54 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>14329</v>
+        <v>14395</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>13135</v>
+        <v>13195</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>10750</v>
+        <v>10796</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>14329</v>
+        <v>14395</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>13135</v>
+        <v>13195</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>10750</v>
+        <v>10796</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>14329</v>
+        <v>14395</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>13135</v>
+        <v>13195</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>10750</v>
+        <v>10796</v>
       </c>
       <c r="O2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-27 20:58:49</t>
+          <t>2026-10-28 17:46:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -602,54 +602,54 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>14275</v>
+        <v>14329</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>13085</v>
+        <v>13135</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>10705</v>
+        <v>10750</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>14275</v>
+        <v>14329</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>13085</v>
+        <v>13135</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>10705</v>
+        <v>10750</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>14275</v>
+        <v>14329</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>13085</v>
+        <v>13135</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>10705</v>
+        <v>10750</v>
       </c>
       <c r="O3" t="n">
         <v>2</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-10-26 21:44:41</t>
+          <t>2026-10-27 20:58:49</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -658,48 +658,54 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>10695</v>
-      </c>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
+        <v>10705</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="I4" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>10695</v>
+        <v>10705</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>10695</v>
+        <v>10705</v>
       </c>
       <c r="O4" t="n">
         <v>2</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-10-25 19:18:46</t>
+          <t>2026-10-26 21:44:41</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -716,15 +722,9 @@
       <c r="E5" s="2" t="n">
         <v>10695</v>
       </c>
-      <c r="F5" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H5" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
       <c r="I5" s="2" t="n">
         <v>14258</v>
       </c>
@@ -748,14 +748,14 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-10-24 18:56:58</t>
+          <t>2026-10-25 19:18:46</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -764,54 +764,54 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-190</v>
+        <v>10</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-175</v>
+        <v>10</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>-145</v>
+        <v>5</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="O6" t="n">
         <v>2</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:04</t>
+          <t>2026-10-24 18:56:58</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -820,54 +820,54 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-170</v>
+        <v>-190</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-155</v>
+        <v>-175</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>-135</v>
+        <v>-145</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="O7" t="n">
         <v>2</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-10-22 20:06:02</t>
+          <t>2026-10-23 19:50:04</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -876,54 +876,54 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-109</v>
+        <v>-170</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-100</v>
+        <v>-155</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>-115</v>
+        <v>-135</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="O8" t="n">
         <v>2</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-10-21 20:04:26</t>
+          <t>2026-10-22 20:06:02</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -932,54 +932,54 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-87</v>
+        <v>-109</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>-80</v>
+        <v>-100</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>-70</v>
+        <v>-115</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="O9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-10-20 23:40:06</t>
+          <t>2026-10-21 20:04:26</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -988,46 +988,54 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="E10" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="F10" s="3" t="n">
-        <v>38</v>
+        <v>-87</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="H10" s="3" t="n"/>
+        <v>-80</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>-70</v>
+      </c>
       <c r="I10" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="K10" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="L10" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="N10" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="O10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-10-19 00:00:00</t>
+          <t>2026-10-20 23:40:06</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1036,31 +1044,31 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="N11" s="2" t="n"/>
       <c r="O11" t="n">
@@ -1068,14 +1076,14 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-10-18 00:00:00</t>
+          <t>2026-10-19 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1091,10 +1099,10 @@
       </c>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="3" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="2" t="n">
@@ -1116,14 +1124,14 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2026-10-17 00:00:00</t>
+          <t>2026-10-18 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1132,31 +1140,31 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="E13" s="2" t="n"/>
       <c r="F13" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="N13" s="2" t="n"/>
       <c r="O13" t="n">
@@ -1164,14 +1172,14 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2026-10-16 00:00:00</t>
+          <t>2026-10-17 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1187,10 +1195,10 @@
       </c>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="3" t="n">
-        <v>-82</v>
+        <v>0</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>-75</v>
+        <v>0</v>
       </c>
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="2" t="n">
@@ -1212,14 +1220,14 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-16 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1228,31 +1236,31 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="3" t="n">
-        <v>-103</v>
+        <v>-82</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-95</v>
+        <v>-75</v>
       </c>
       <c r="H15" s="3" t="n"/>
       <c r="I15" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="N15" s="2" t="n"/>
       <c r="O15" t="n">
@@ -1260,14 +1268,14 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1276,31 +1284,31 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="3" t="n">
-        <v>-39</v>
+        <v>-103</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>-35</v>
+        <v>-95</v>
       </c>
       <c r="H16" s="3" t="n"/>
       <c r="I16" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="N16" s="2" t="n"/>
       <c r="O16" t="n">
@@ -1308,14 +1316,14 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1324,31 +1332,31 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="3" t="n">
-        <v>-174</v>
+        <v>-39</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>-160</v>
+        <v>-35</v>
       </c>
       <c r="H17" s="3" t="n"/>
       <c r="I17" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="N17" s="2" t="n"/>
       <c r="O17" t="n">
@@ -1356,14 +1364,14 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>2026-10-12 00:00:00</t>
+          <t>2026-10-13 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1372,37 +1380,85 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="3" t="n">
-        <v>0</v>
+        <v>-174</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>0</v>
+        <v>-160</v>
       </c>
       <c r="H18" s="3" t="n"/>
       <c r="I18" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="N18" s="2" t="n"/>
       <c r="O18" t="n">
         <v>1</v>
       </c>
       <c r="P18" t="inlineStr">
+        <is>
+          <t>2026-10-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="3" t="n"/>
+      <c r="I19" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="N19" s="2" t="n"/>
+      <c r="O19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P19" t="inlineStr">
         <is>
           <t>2026-10-11 00:00:00</t>
         </is>
@@ -1419,7 +1475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4786,6 +4842,150 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-10-28 17:46:54</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="n">
+        <v>14395</v>
+      </c>
+      <c r="H71" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-10-28 17:46:54</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="n">
+        <v>13195</v>
+      </c>
+      <c r="H72" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-10-28 17:46:54</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="n">
+        <v>10796</v>
+      </c>
+      <c r="H73" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-28 21:41 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -582,11 +582,11 @@
         <v>10796</v>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-28 17:46:54</t>
+          <t>2026-10-28 21:41:44</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4986,6 +4986,150 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-10-28 21:41:44</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>14395</v>
+      </c>
+      <c r="H74" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-10-28 21:41:44</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="n">
+        <v>13195</v>
+      </c>
+      <c r="H75" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-10-28 21:41:44</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>10796</v>
+      </c>
+      <c r="H76" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-29 17:56 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -554,15 +554,9 @@
       <c r="E2" s="2" t="n">
         <v>10796</v>
       </c>
-      <c r="F2" s="3" t="n">
-        <v>66</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>60</v>
-      </c>
-      <c r="H2" s="3" t="n">
-        <v>46</v>
-      </c>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
       <c r="I2" s="2" t="n">
         <v>14395</v>
       </c>
@@ -582,18 +576,18 @@
         <v>10796</v>
       </c>
       <c r="O2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-28 21:41:44</t>
+          <t>2026-10-29 17:56:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -602,54 +596,54 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>14329</v>
+        <v>14395</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>13135</v>
+        <v>13195</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>10750</v>
+        <v>10796</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>14329</v>
+        <v>14395</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>13135</v>
+        <v>13195</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>10750</v>
+        <v>10796</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>14329</v>
+        <v>14395</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>13135</v>
+        <v>13195</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>10750</v>
+        <v>10796</v>
       </c>
       <c r="O3" t="n">
         <v>2</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-10-27 20:58:49</t>
+          <t>2026-10-28 21:41:44</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -658,54 +652,54 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>14275</v>
+        <v>14329</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>13085</v>
+        <v>13135</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>10705</v>
+        <v>10750</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>14275</v>
+        <v>14329</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>13085</v>
+        <v>13135</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>10705</v>
+        <v>10750</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>14275</v>
+        <v>14329</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>13085</v>
+        <v>13135</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>10705</v>
+        <v>10750</v>
       </c>
       <c r="O4" t="n">
         <v>2</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-10-26 21:44:41</t>
+          <t>2026-10-27 20:58:49</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -714,48 +708,54 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10695</v>
-      </c>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
+        <v>10705</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="I5" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>10695</v>
+        <v>10705</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>10695</v>
+        <v>10705</v>
       </c>
       <c r="O5" t="n">
         <v>2</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-10-25 19:18:46</t>
+          <t>2026-10-26 21:44:41</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -772,15 +772,9 @@
       <c r="E6" s="2" t="n">
         <v>10695</v>
       </c>
-      <c r="F6" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H6" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
       <c r="I6" s="2" t="n">
         <v>14258</v>
       </c>
@@ -804,14 +798,14 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-10-24 18:56:58</t>
+          <t>2026-10-25 19:18:46</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -820,54 +814,54 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-190</v>
+        <v>10</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-175</v>
+        <v>10</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>-145</v>
+        <v>5</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="O7" t="n">
         <v>2</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:04</t>
+          <t>2026-10-24 18:56:58</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -876,54 +870,54 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-170</v>
+        <v>-190</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-155</v>
+        <v>-175</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>-135</v>
+        <v>-145</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="O8" t="n">
         <v>2</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-10-22 20:06:02</t>
+          <t>2026-10-23 19:50:04</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -932,54 +926,54 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-109</v>
+        <v>-170</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>-100</v>
+        <v>-155</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>-115</v>
+        <v>-135</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="O9" t="n">
         <v>2</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-10-21 20:04:26</t>
+          <t>2026-10-22 20:06:02</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -988,54 +982,54 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-87</v>
+        <v>-109</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-80</v>
+        <v>-100</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>-70</v>
+        <v>-115</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="O10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-10-20 23:40:06</t>
+          <t>2026-10-21 20:04:26</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1044,46 +1038,54 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="E11" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="F11" s="3" t="n">
-        <v>38</v>
+        <v>-87</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="H11" s="3" t="n"/>
+        <v>-80</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>-70</v>
+      </c>
       <c r="I11" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="K11" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="L11" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="N11" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="O11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-10-19 00:00:00</t>
+          <t>2026-10-20 23:40:06</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1092,31 +1094,31 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="N12" s="2" t="n"/>
       <c r="O12" t="n">
@@ -1124,14 +1126,14 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2026-10-18 00:00:00</t>
+          <t>2026-10-19 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1147,10 +1149,10 @@
       </c>
       <c r="E13" s="2" t="n"/>
       <c r="F13" s="3" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="2" t="n">
@@ -1172,14 +1174,14 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2026-10-17 00:00:00</t>
+          <t>2026-10-18 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1188,31 +1190,31 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="N14" s="2" t="n"/>
       <c r="O14" t="n">
@@ -1220,14 +1222,14 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2026-10-16 00:00:00</t>
+          <t>2026-10-17 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1243,10 +1245,10 @@
       </c>
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="3" t="n">
-        <v>-82</v>
+        <v>0</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-75</v>
+        <v>0</v>
       </c>
       <c r="H15" s="3" t="n"/>
       <c r="I15" s="2" t="n">
@@ -1268,14 +1270,14 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-16 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1284,31 +1286,31 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="3" t="n">
-        <v>-103</v>
+        <v>-82</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>-95</v>
+        <v>-75</v>
       </c>
       <c r="H16" s="3" t="n"/>
       <c r="I16" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="N16" s="2" t="n"/>
       <c r="O16" t="n">
@@ -1316,14 +1318,14 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1332,31 +1334,31 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="3" t="n">
-        <v>-39</v>
+        <v>-103</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>-35</v>
+        <v>-95</v>
       </c>
       <c r="H17" s="3" t="n"/>
       <c r="I17" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="N17" s="2" t="n"/>
       <c r="O17" t="n">
@@ -1364,14 +1366,14 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1380,31 +1382,31 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="3" t="n">
-        <v>-174</v>
+        <v>-39</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>-160</v>
+        <v>-35</v>
       </c>
       <c r="H18" s="3" t="n"/>
       <c r="I18" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="N18" s="2" t="n"/>
       <c r="O18" t="n">
@@ -1412,14 +1414,14 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2026-10-12 00:00:00</t>
+          <t>2026-10-13 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1428,37 +1430,85 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="3" t="n">
-        <v>0</v>
+        <v>-174</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>0</v>
+        <v>-160</v>
       </c>
       <c r="H19" s="3" t="n"/>
       <c r="I19" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="K19" s="2" t="n"/>
       <c r="L19" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="N19" s="2" t="n"/>
       <c r="O19" t="n">
         <v>1</v>
       </c>
       <c r="P19" t="inlineStr">
+        <is>
+          <t>2026-10-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="3" t="n"/>
+      <c r="I20" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="N20" s="2" t="n"/>
+      <c r="O20" t="n">
+        <v>1</v>
+      </c>
+      <c r="P20" t="inlineStr">
         <is>
           <t>2026-10-11 00:00:00</t>
         </is>
@@ -1475,7 +1525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5130,6 +5180,144 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-10-29 17:56:13</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>14395</v>
+      </c>
+      <c r="H77" s="3" t="n"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-10-29 17:56:13</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="n">
+        <v>13195</v>
+      </c>
+      <c r="H78" s="3" t="n"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-10-29 17:56:13</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="n">
+        <v>10796</v>
+      </c>
+      <c r="H79" s="3" t="n"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-29 21:48 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -576,11 +576,11 @@
         <v>10796</v>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:56:13</t>
+          <t>2026-10-29 21:48:24</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:J82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5318,6 +5318,144 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-10-29 21:48:24</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="n">
+        <v>14395</v>
+      </c>
+      <c r="H80" s="3" t="n"/>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-10-29 21:48:24</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="n">
+        <v>13195</v>
+      </c>
+      <c r="H81" s="3" t="n"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-10-29 21:48:24</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="n">
+        <v>10796</v>
+      </c>
+      <c r="H82" s="3" t="n"/>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-30 17:47 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -546,48 +546,54 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>14395</v>
+        <v>14226</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>13195</v>
+        <v>13040</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>10796</v>
-      </c>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
+        <v>10667</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>-169</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>-155</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>-129</v>
+      </c>
       <c r="I2" s="2" t="n">
-        <v>14395</v>
+        <v>14226</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>13195</v>
+        <v>13040</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>10796</v>
+        <v>10667</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>14395</v>
+        <v>14226</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>13195</v>
+        <v>13040</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>10796</v>
+        <v>10667</v>
       </c>
       <c r="O2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:48:24</t>
+          <t>2026-10-30 17:47:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -604,15 +610,9 @@
       <c r="E3" s="2" t="n">
         <v>10796</v>
       </c>
-      <c r="F3" s="3" t="n">
-        <v>66</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>60</v>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>46</v>
-      </c>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
       <c r="I3" s="2" t="n">
         <v>14395</v>
       </c>
@@ -636,14 +636,14 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-10-28 21:41:44</t>
+          <t>2026-10-29 21:48:24</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -652,54 +652,54 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>14329</v>
+        <v>14395</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>13135</v>
+        <v>13195</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>10750</v>
+        <v>10796</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>14329</v>
+        <v>14395</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>13135</v>
+        <v>13195</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>10750</v>
+        <v>10796</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>14329</v>
+        <v>14395</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>13135</v>
+        <v>13195</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>10750</v>
+        <v>10796</v>
       </c>
       <c r="O4" t="n">
         <v>2</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-10-27 20:58:49</t>
+          <t>2026-10-28 21:41:44</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -708,54 +708,54 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>14275</v>
+        <v>14329</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>13085</v>
+        <v>13135</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10705</v>
+        <v>10750</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>14275</v>
+        <v>14329</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>13085</v>
+        <v>13135</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>10705</v>
+        <v>10750</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>14275</v>
+        <v>14329</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>13085</v>
+        <v>13135</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>10705</v>
+        <v>10750</v>
       </c>
       <c r="O5" t="n">
         <v>2</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-10-26 21:44:41</t>
+          <t>2026-10-27 20:58:49</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -764,48 +764,54 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>10695</v>
-      </c>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
+        <v>10705</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="I6" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>10695</v>
+        <v>10705</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>10695</v>
+        <v>10705</v>
       </c>
       <c r="O6" t="n">
         <v>2</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-10-25 19:18:46</t>
+          <t>2026-10-26 21:44:41</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -822,15 +828,9 @@
       <c r="E7" s="2" t="n">
         <v>10695</v>
       </c>
-      <c r="F7" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
       <c r="I7" s="2" t="n">
         <v>14258</v>
       </c>
@@ -854,14 +854,14 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-10-24 18:56:58</t>
+          <t>2026-10-25 19:18:46</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -870,54 +870,54 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-190</v>
+        <v>10</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>-175</v>
+        <v>10</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>-145</v>
+        <v>5</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="O8" t="n">
         <v>2</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:04</t>
+          <t>2026-10-24 18:56:58</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -926,54 +926,54 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-170</v>
+        <v>-190</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>-155</v>
+        <v>-175</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>-135</v>
+        <v>-145</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="O9" t="n">
         <v>2</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-10-22 20:06:02</t>
+          <t>2026-10-23 19:50:04</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -982,54 +982,54 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-109</v>
+        <v>-170</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-100</v>
+        <v>-155</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>-115</v>
+        <v>-135</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="O10" t="n">
         <v>2</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-10-21 20:04:26</t>
+          <t>2026-10-22 20:06:02</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1038,54 +1038,54 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>-87</v>
+        <v>-109</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>-80</v>
+        <v>-100</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>-70</v>
+        <v>-115</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="O11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-10-20 23:40:06</t>
+          <t>2026-10-21 20:04:26</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1094,46 +1094,54 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="E12" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="F12" s="3" t="n">
-        <v>38</v>
+        <v>-87</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="H12" s="3" t="n"/>
+        <v>-80</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>-70</v>
+      </c>
       <c r="I12" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="K12" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="L12" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="N12" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="O12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2026-10-19 00:00:00</t>
+          <t>2026-10-20 23:40:06</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1142,31 +1150,31 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="E13" s="2" t="n"/>
       <c r="F13" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="N13" s="2" t="n"/>
       <c r="O13" t="n">
@@ -1174,14 +1182,14 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2026-10-18 00:00:00</t>
+          <t>2026-10-19 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1197,10 +1205,10 @@
       </c>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="3" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="2" t="n">
@@ -1222,14 +1230,14 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2026-10-17 00:00:00</t>
+          <t>2026-10-18 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1238,31 +1246,31 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H15" s="3" t="n"/>
       <c r="I15" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="N15" s="2" t="n"/>
       <c r="O15" t="n">
@@ -1270,14 +1278,14 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2026-10-16 00:00:00</t>
+          <t>2026-10-17 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1293,10 +1301,10 @@
       </c>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="3" t="n">
-        <v>-82</v>
+        <v>0</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>-75</v>
+        <v>0</v>
       </c>
       <c r="H16" s="3" t="n"/>
       <c r="I16" s="2" t="n">
@@ -1318,14 +1326,14 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-16 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1334,31 +1342,31 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="3" t="n">
-        <v>-103</v>
+        <v>-82</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>-95</v>
+        <v>-75</v>
       </c>
       <c r="H17" s="3" t="n"/>
       <c r="I17" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="N17" s="2" t="n"/>
       <c r="O17" t="n">
@@ -1366,14 +1374,14 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1382,31 +1390,31 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="3" t="n">
-        <v>-39</v>
+        <v>-103</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>-35</v>
+        <v>-95</v>
       </c>
       <c r="H18" s="3" t="n"/>
       <c r="I18" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="N18" s="2" t="n"/>
       <c r="O18" t="n">
@@ -1414,14 +1422,14 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1430,31 +1438,31 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="3" t="n">
-        <v>-174</v>
+        <v>-39</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>-160</v>
+        <v>-35</v>
       </c>
       <c r="H19" s="3" t="n"/>
       <c r="I19" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="K19" s="2" t="n"/>
       <c r="L19" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="N19" s="2" t="n"/>
       <c r="O19" t="n">
@@ -1462,14 +1470,14 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2026-10-12 00:00:00</t>
+          <t>2026-10-13 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1478,37 +1486,85 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="3" t="n">
-        <v>0</v>
+        <v>-174</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>0</v>
+        <v>-160</v>
       </c>
       <c r="H20" s="3" t="n"/>
       <c r="I20" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="K20" s="2" t="n"/>
       <c r="L20" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="N20" s="2" t="n"/>
       <c r="O20" t="n">
         <v>1</v>
       </c>
       <c r="P20" t="inlineStr">
+        <is>
+          <t>2026-10-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="3" t="n"/>
+      <c r="I21" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="K21" s="2" t="n"/>
+      <c r="L21" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="N21" s="2" t="n"/>
+      <c r="O21" t="n">
+        <v>1</v>
+      </c>
+      <c r="P21" t="inlineStr">
         <is>
           <t>2026-10-11 00:00:00</t>
         </is>
@@ -1525,7 +1581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J82"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5456,6 +5512,150 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:47:39</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="n">
+        <v>14226</v>
+      </c>
+      <c r="H83" s="3" t="n">
+        <v>-169</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:47:39</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="n">
+        <v>13040</v>
+      </c>
+      <c r="H84" s="3" t="n">
+        <v>-155</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:47:39</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="n">
+        <v>10667</v>
+      </c>
+      <c r="H85" s="3" t="n">
+        <v>-129</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-30 21:37 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -582,11 +582,11 @@
         <v>10667</v>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:47:39</t>
+          <t>2026-10-30 21:37:22</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5656,6 +5656,150 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-10-30 21:37:22</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="n">
+        <v>14226</v>
+      </c>
+      <c r="H86" s="3" t="n">
+        <v>-169</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-10-30 21:37:22</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="n">
+        <v>13040</v>
+      </c>
+      <c r="H87" s="3" t="n">
+        <v>-155</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-10-30 21:37:22</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="n">
+        <v>10667</v>
+      </c>
+      <c r="H88" s="3" t="n">
+        <v>-129</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-31 17:19 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -546,54 +546,54 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>14226</v>
+        <v>13888</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>13040</v>
+        <v>12730</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>10667</v>
+        <v>10416</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-169</v>
+        <v>-338</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-155</v>
+        <v>-310</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>-129</v>
+        <v>-251</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>14226</v>
+        <v>13888</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>13040</v>
+        <v>12730</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>10667</v>
+        <v>10416</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>14226</v>
+        <v>13888</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>13040</v>
+        <v>12730</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>10667</v>
+        <v>10416</v>
       </c>
       <c r="O2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-30 21:37:22</t>
+          <t>2026-10-31 17:19:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -602,48 +602,54 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>14395</v>
+        <v>14226</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>13195</v>
+        <v>13040</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>10796</v>
-      </c>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
+        <v>10667</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>-169</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>-155</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>-129</v>
+      </c>
       <c r="I3" s="2" t="n">
-        <v>14395</v>
+        <v>14226</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>13195</v>
+        <v>13040</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>10796</v>
+        <v>10667</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>14395</v>
+        <v>14226</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>13195</v>
+        <v>13040</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>10796</v>
+        <v>10667</v>
       </c>
       <c r="O3" t="n">
         <v>2</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-10-29 21:48:24</t>
+          <t>2026-10-30 21:37:22</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -660,15 +666,9 @@
       <c r="E4" s="2" t="n">
         <v>10796</v>
       </c>
-      <c r="F4" s="3" t="n">
-        <v>66</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>60</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>46</v>
-      </c>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
       <c r="I4" s="2" t="n">
         <v>14395</v>
       </c>
@@ -692,14 +692,14 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-10-28 21:41:44</t>
+          <t>2026-10-29 21:48:24</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -708,54 +708,54 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>14329</v>
+        <v>14395</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>13135</v>
+        <v>13195</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10750</v>
+        <v>10796</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>14329</v>
+        <v>14395</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>13135</v>
+        <v>13195</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>10750</v>
+        <v>10796</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>14329</v>
+        <v>14395</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>13135</v>
+        <v>13195</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>10750</v>
+        <v>10796</v>
       </c>
       <c r="O5" t="n">
         <v>2</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-10-27 20:58:49</t>
+          <t>2026-10-28 21:41:44</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -764,54 +764,54 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>14275</v>
+        <v>14329</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>13085</v>
+        <v>13135</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>10705</v>
+        <v>10750</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>14275</v>
+        <v>14329</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>13085</v>
+        <v>13135</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>10705</v>
+        <v>10750</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>14275</v>
+        <v>14329</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>13085</v>
+        <v>13135</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>10705</v>
+        <v>10750</v>
       </c>
       <c r="O6" t="n">
         <v>2</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-10-26 21:44:41</t>
+          <t>2026-10-27 20:58:49</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -820,48 +820,54 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>10695</v>
-      </c>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
+        <v>10705</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>10</v>
+      </c>
       <c r="I7" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>10695</v>
+        <v>10705</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>14258</v>
+        <v>14275</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>13070</v>
+        <v>13085</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>10695</v>
+        <v>10705</v>
       </c>
       <c r="O7" t="n">
         <v>2</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-10-25 19:18:46</t>
+          <t>2026-10-26 21:44:41</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -878,15 +884,9 @@
       <c r="E8" s="2" t="n">
         <v>10695</v>
       </c>
-      <c r="F8" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="G8" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H8" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
       <c r="I8" s="2" t="n">
         <v>14258</v>
       </c>
@@ -910,14 +910,14 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-10-24 18:56:58</t>
+          <t>2026-10-25 19:18:46</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -926,54 +926,54 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-190</v>
+        <v>10</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>-175</v>
+        <v>10</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>-145</v>
+        <v>5</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>14248</v>
+        <v>14258</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>13060</v>
+        <v>13070</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>10690</v>
+        <v>10695</v>
       </c>
       <c r="O9" t="n">
         <v>2</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:04</t>
+          <t>2026-10-24 18:56:58</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -982,54 +982,54 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-170</v>
+        <v>-190</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-155</v>
+        <v>-175</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>-135</v>
+        <v>-145</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>14438</v>
+        <v>14248</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>13235</v>
+        <v>13060</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>10835</v>
+        <v>10690</v>
       </c>
       <c r="O10" t="n">
         <v>2</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-10-22 20:06:02</t>
+          <t>2026-10-23 19:50:04</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1038,54 +1038,54 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>-109</v>
+        <v>-170</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>-100</v>
+        <v>-155</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>-115</v>
+        <v>-135</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>14608</v>
+        <v>14438</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>13390</v>
+        <v>13235</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>10970</v>
+        <v>10835</v>
       </c>
       <c r="O11" t="n">
         <v>2</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-10-21 20:04:26</t>
+          <t>2026-10-22 20:06:02</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1094,54 +1094,54 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-87</v>
+        <v>-109</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-80</v>
+        <v>-100</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>-70</v>
+        <v>-115</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>14717</v>
+        <v>14608</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>13490</v>
+        <v>13390</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>11085</v>
+        <v>10970</v>
       </c>
       <c r="O12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2026-10-20 23:40:06</t>
+          <t>2026-10-21 20:04:26</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1150,46 +1150,54 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="E13" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="F13" s="3" t="n">
-        <v>38</v>
+        <v>-87</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="H13" s="3" t="n"/>
+        <v>-80</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>-70</v>
+      </c>
       <c r="I13" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="K13" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="L13" s="2" t="n">
-        <v>14804</v>
+        <v>14717</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>13570</v>
-      </c>
-      <c r="N13" s="2" t="n"/>
+        <v>13490</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>11085</v>
+      </c>
       <c r="O13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2026-10-19 00:00:00</t>
+          <t>2026-10-20 23:40:06</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1198,31 +1206,31 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="3" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n">
-        <v>14766</v>
+        <v>14804</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>13535</v>
+        <v>13570</v>
       </c>
       <c r="N14" s="2" t="n"/>
       <c r="O14" t="n">
@@ -1230,14 +1238,14 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2026-10-18 00:00:00</t>
+          <t>2026-10-19 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1253,10 +1261,10 @@
       </c>
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="3" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H15" s="3" t="n"/>
       <c r="I15" s="2" t="n">
@@ -1278,14 +1286,14 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2026-10-17 00:00:00</t>
+          <t>2026-10-18 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1294,31 +1302,31 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H16" s="3" t="n"/>
       <c r="I16" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n">
-        <v>14744</v>
+        <v>14766</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>13515</v>
+        <v>13535</v>
       </c>
       <c r="N16" s="2" t="n"/>
       <c r="O16" t="n">
@@ -1326,14 +1334,14 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>2026-10-16 00:00:00</t>
+          <t>2026-10-17 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1349,10 +1357,10 @@
       </c>
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="3" t="n">
-        <v>-82</v>
+        <v>0</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>-75</v>
+        <v>0</v>
       </c>
       <c r="H17" s="3" t="n"/>
       <c r="I17" s="2" t="n">
@@ -1374,14 +1382,14 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>2026-10-15 00:00:00</t>
+          <t>2026-10-16 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1390,31 +1398,31 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="3" t="n">
-        <v>-103</v>
+        <v>-82</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>-95</v>
+        <v>-75</v>
       </c>
       <c r="H18" s="3" t="n"/>
       <c r="I18" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n">
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>13590</v>
+        <v>13515</v>
       </c>
       <c r="N18" s="2" t="n"/>
       <c r="O18" t="n">
@@ -1422,14 +1430,14 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2026-10-14 00:00:00</t>
+          <t>2026-10-15 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1438,31 +1446,31 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="3" t="n">
-        <v>-39</v>
+        <v>-103</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>-35</v>
+        <v>-95</v>
       </c>
       <c r="H19" s="3" t="n"/>
       <c r="I19" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="K19" s="2" t="n"/>
       <c r="L19" s="2" t="n">
-        <v>14929</v>
+        <v>14826</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>13685</v>
+        <v>13590</v>
       </c>
       <c r="N19" s="2" t="n"/>
       <c r="O19" t="n">
@@ -1470,14 +1478,14 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2026-10-13 00:00:00</t>
+          <t>2026-10-14 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1486,31 +1494,31 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="3" t="n">
-        <v>-174</v>
+        <v>-39</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>-160</v>
+        <v>-35</v>
       </c>
       <c r="H20" s="3" t="n"/>
       <c r="I20" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="K20" s="2" t="n"/>
       <c r="L20" s="2" t="n">
-        <v>14968</v>
+        <v>14929</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>13720</v>
+        <v>13685</v>
       </c>
       <c r="N20" s="2" t="n"/>
       <c r="O20" t="n">
@@ -1518,14 +1526,14 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>2026-10-12 00:00:00</t>
+          <t>2026-10-13 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1534,37 +1542,85 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="E21" s="2" t="n"/>
       <c r="F21" s="3" t="n">
-        <v>0</v>
+        <v>-174</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>0</v>
+        <v>-160</v>
       </c>
       <c r="H21" s="3" t="n"/>
       <c r="I21" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="K21" s="2" t="n"/>
       <c r="L21" s="2" t="n">
-        <v>15142</v>
+        <v>14968</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>13880</v>
+        <v>13720</v>
       </c>
       <c r="N21" s="2" t="n"/>
       <c r="O21" t="n">
         <v>1</v>
       </c>
       <c r="P21" t="inlineStr">
+        <is>
+          <t>2026-10-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="3" t="n"/>
+      <c r="I22" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="n">
+        <v>15142</v>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>13880</v>
+      </c>
+      <c r="N22" s="2" t="n"/>
+      <c r="O22" t="n">
+        <v>1</v>
+      </c>
+      <c r="P22" t="inlineStr">
         <is>
           <t>2026-10-11 00:00:00</t>
         </is>
@@ -1581,7 +1637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5800,6 +5856,150 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-10-31 17:19:11</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="n">
+        <v>13888</v>
+      </c>
+      <c r="H89" s="3" t="n">
+        <v>-338</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-10-31 17:19:11</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="n">
+        <v>12730</v>
+      </c>
+      <c r="H90" s="3" t="n">
+        <v>-310</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-10-31 17:19:11</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="n">
+        <v>10416</v>
+      </c>
+      <c r="H91" s="3" t="n">
+        <v>-251</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rates update 2026-10-31 20:57 IST
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -582,11 +582,11 @@
         <v>10416</v>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-31 17:19:11</t>
+          <t>2026-10-31 20:57:16</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J91"/>
+  <dimension ref="A1:J94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6000,6 +6000,150 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-10-31 20:57:16</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>24K</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="n">
+        <v>13888</v>
+      </c>
+      <c r="H92" s="3" t="n">
+        <v>-338</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-10-31 20:57:16</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>22K</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="n">
+        <v>12730</v>
+      </c>
+      <c r="H93" s="3" t="n">
+        <v>-310</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-10-31 20:57:16</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>18K</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="n">
+        <v>10416</v>
+      </c>
+      <c r="H94" s="3" t="n">
+        <v>-251</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>https://www.goodreturns.in/gold-rates/chennai.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>